<commit_message>
refactor: introduce cross-section percentile ranking function and update related logic in analysis scripts; enhance run_meta.json with new regressor descriptions for clarity
</commit_message>
<xml_diff>
--- a/outputs/05_benchmark_signals/tables_v_viii/cn/table_vi_forecast_logit.xlsx
+++ b/outputs/05_benchmark_signals/tables_v_viii/cn/table_vi_forecast_logit.xlsx
@@ -442,17 +442,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.00 (0.4)</t>
+          <t>0.01 (0.1)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.00** (2.2)</t>
+          <t>0.16*** (2.8)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.00* (1.7)</t>
+          <t>0.14** (2.2)</t>
         </is>
       </c>
     </row>
@@ -464,17 +464,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.00*** (3.0)</t>
+          <t>0.24*** (3.1)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-0.00 (-0.3)</t>
+          <t>-0.03 (-0.2)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.00* (2.0)</t>
+          <t>0.17** (2.1)</t>
         </is>
       </c>
     </row>
@@ -486,17 +486,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.00*** (8.8)</t>
+          <t>1.17*** (9.2)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.00*** (5.2)</t>
+          <t>0.77*** (7.4)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.00*** (4.2)</t>
+          <t>0.48*** (5.9)</t>
         </is>
       </c>
     </row>
@@ -508,17 +508,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-0.00 (-1.0)</t>
+          <t>-0.26 (-1.2)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.00 (0.5)</t>
+          <t>0.04 (0.2)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.00 (-0.4)</t>
+          <t>-0.08 (-0.8)</t>
         </is>
       </c>
     </row>
@@ -530,17 +530,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.00*** (5.0)</t>
+          <t>0.53*** (5.1)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.00*** (3.2)</t>
+          <t>0.32*** (3.8)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.00*** (3.4)</t>
+          <t>0.44*** (4.0)</t>
         </is>
       </c>
     </row>
@@ -552,17 +552,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>-0.00 (-1.0)</t>
+          <t>-0.07 (-1.0)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>-0.00 (-0.2)</t>
+          <t>-0.17 (-1.1)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.00*** (-3.1)</t>
+          <t>-0.28*** (-3.2)</t>
         </is>
       </c>
     </row>
@@ -574,17 +574,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>-0.00 (-0.7)</t>
+          <t>-0.07 (-0.7)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.00 (0.9)</t>
+          <t>0.06 (0.7)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.00 (1.1)</t>
+          <t>0.10 (1.1)</t>
         </is>
       </c>
     </row>
@@ -596,17 +596,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-0.00*** (-4.1)</t>
+          <t>-0.86*** (-4.4)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>-0.00*** (-5.2)</t>
+          <t>-0.68*** (-4.9)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.00*** (-4.3)</t>
+          <t>-0.54*** (-5.6)</t>
         </is>
       </c>
     </row>
@@ -618,17 +618,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0.00*** (9.1)</t>
+          <t>0.52*** (8.6)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.00*** (4.5)</t>
+          <t>0.31*** (5.3)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.00*** (2.9)</t>
+          <t>0.18*** (2.9)</t>
         </is>
       </c>
     </row>
@@ -640,17 +640,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.00*** (3.7)</t>
+          <t>0.21*** (3.7)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-0.00** (-2.1)</t>
+          <t>-0.27*** (-2.8)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.00 (1.5)</t>
+          <t>0.11* (1.8)</t>
         </is>
       </c>
     </row>
@@ -662,17 +662,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>-0.00*** (-4.7)</t>
+          <t>-0.98*** (-4.9)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-0.00*** (-3.7)</t>
+          <t>-0.73*** (-5.0)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.00** (-2.4)</t>
+          <t>-0.26** (-2.4)</t>
         </is>
       </c>
     </row>
@@ -684,17 +684,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.00*** (3.0)</t>
+          <t>-0.13 (-1.1)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.00** (2.0)</t>
+          <t>-0.15** (-2.1)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.00 (1.0)</t>
+          <t>-0.12** (-2.1)</t>
         </is>
       </c>
     </row>
@@ -706,17 +706,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>2.52</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1.05</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>1.14</t>
         </is>
       </c>
     </row>
@@ -773,22 +773,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.279727903468155e-05</v>
+        <v>0.005133628793717287</v>
       </c>
       <c r="C2" t="n">
-        <v>6.584624253434957e-05</v>
+        <v>0.1587720828178919</v>
       </c>
       <c r="D2" t="n">
-        <v>5.62971386565906e-05</v>
+        <v>0.1412781253809955</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3777365528233277</v>
+        <v>0.07789742659940276</v>
       </c>
       <c r="F2" t="n">
-        <v>2.155550571266879</v>
+        <v>2.777129763598408</v>
       </c>
       <c r="G2" t="n">
-        <v>1.672626877915041</v>
+        <v>2.158410008997297</v>
       </c>
     </row>
     <row r="3">
@@ -798,22 +798,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0001144825937718384</v>
+        <v>0.2434323672665021</v>
       </c>
       <c r="C3" t="n">
-        <v>-2.736313962500434e-05</v>
+        <v>-0.03284989593887466</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0001005349567761181</v>
+        <v>0.1653277710832319</v>
       </c>
       <c r="E3" t="n">
-        <v>3.02510515326343</v>
+        <v>3.09596502926108</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.3103908232304647</v>
+        <v>-0.201759430720532</v>
       </c>
       <c r="G3" t="n">
-        <v>1.956459547382654</v>
+        <v>2.052149705526685</v>
       </c>
     </row>
     <row r="4">
@@ -823,22 +823,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0009076060321783584</v>
+        <v>1.169127408648351</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0006079463372253088</v>
+        <v>0.7712371901269278</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0003715427544615843</v>
+        <v>0.4797511413237523</v>
       </c>
       <c r="E4" t="n">
-        <v>8.798132970657514</v>
+        <v>9.229415976909975</v>
       </c>
       <c r="F4" t="n">
-        <v>5.186913277244475</v>
+        <v>7.422619741785581</v>
       </c>
       <c r="G4" t="n">
-        <v>4.19390391429625</v>
+        <v>5.929478540993649</v>
       </c>
     </row>
     <row r="5">
@@ -848,22 +848,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-0.0001033943393676158</v>
+        <v>-0.2599308325373778</v>
       </c>
       <c r="C5" t="n">
-        <v>5.187911653772215e-05</v>
+        <v>0.03887555302521005</v>
       </c>
       <c r="D5" t="n">
-        <v>-2.702293294480636e-05</v>
+        <v>-0.08110230628937461</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.9779860670382932</v>
+        <v>-1.246530661352819</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4992087510442095</v>
+        <v>0.2176932446738779</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.4301149955207051</v>
+        <v>-0.7629483527505903</v>
       </c>
     </row>
     <row r="6">
@@ -873,22 +873,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0002438091326313685</v>
+        <v>0.5333456072881336</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0001750325529356021</v>
+        <v>0.3216694777696864</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0002404432263079599</v>
+        <v>0.4448986962282541</v>
       </c>
       <c r="E6" t="n">
-        <v>4.961460424904557</v>
+        <v>5.070661080691911</v>
       </c>
       <c r="F6" t="n">
-        <v>3.151581545595518</v>
+        <v>3.815297809327104</v>
       </c>
       <c r="G6" t="n">
-        <v>3.425286816284014</v>
+        <v>4.008012772340785</v>
       </c>
     </row>
     <row r="7">
@@ -898,22 +898,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-3.156454625858023e-05</v>
+        <v>-0.06563103700477606</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.445849221020027e-05</v>
+        <v>-0.1668269908492441</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.0001324732747302813</v>
+        <v>-0.2771208059569606</v>
       </c>
       <c r="E7" t="n">
-        <v>-1.019221495736963</v>
+        <v>-1.022678958450186</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.2499185307657797</v>
+        <v>-1.129933060042729</v>
       </c>
       <c r="G7" t="n">
-        <v>-3.118270927503277</v>
+        <v>-3.219168362357553</v>
       </c>
     </row>
     <row r="8">
@@ -923,22 +923,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-3.233484813223899e-05</v>
+        <v>-0.06786972751477695</v>
       </c>
       <c r="C8" t="n">
-        <v>5.349978416418032e-05</v>
+        <v>0.05854188474986363</v>
       </c>
       <c r="D8" t="n">
-        <v>7.213074030073425e-05</v>
+        <v>0.09932916921514628</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.6756210066743904</v>
+        <v>-0.7154580055617121</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9416786856802982</v>
+        <v>0.6708957872070971</v>
       </c>
       <c r="G8" t="n">
-        <v>1.120519170801434</v>
+        <v>1.097698024596533</v>
       </c>
     </row>
     <row r="9">
@@ -948,22 +948,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-0.0003757471783495751</v>
+        <v>-0.8574385528333964</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.000321911669683012</v>
+        <v>-0.6796447885362304</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.0002792911226729194</v>
+        <v>-0.5362866366753224</v>
       </c>
       <c r="E9" t="n">
-        <v>-4.113257264318539</v>
+        <v>-4.366728670660028</v>
       </c>
       <c r="F9" t="n">
-        <v>-5.237941287335897</v>
+        <v>-4.937035445329859</v>
       </c>
       <c r="G9" t="n">
-        <v>-4.313395903494101</v>
+        <v>-5.559704692425314</v>
       </c>
     </row>
     <row r="10">
@@ -973,22 +973,22 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.000566761810729536</v>
+        <v>0.517980466373016</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0003654078670787664</v>
+        <v>0.3092641542164269</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0002217341913497647</v>
+        <v>0.1802850932607646</v>
       </c>
       <c r="E10" t="n">
-        <v>9.067487804093886</v>
+        <v>8.60816941711408</v>
       </c>
       <c r="F10" t="n">
-        <v>4.500472583538061</v>
+        <v>5.333927134097804</v>
       </c>
       <c r="G10" t="n">
-        <v>2.908083043452617</v>
+        <v>2.914165551391138</v>
       </c>
     </row>
     <row r="11">
@@ -998,22 +998,22 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0001101250516177593</v>
+        <v>0.2103506384673837</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.0001682604037558795</v>
+        <v>-0.2682200711389841</v>
       </c>
       <c r="D11" t="n">
-        <v>4.516337162044826e-05</v>
+        <v>0.110514018718214</v>
       </c>
       <c r="E11" t="n">
-        <v>3.665408709633833</v>
+        <v>3.692972061784666</v>
       </c>
       <c r="F11" t="n">
-        <v>-2.140186314363858</v>
+        <v>-2.799533459717596</v>
       </c>
       <c r="G11" t="n">
-        <v>1.462312400639133</v>
+        <v>1.755635367133506</v>
       </c>
     </row>
     <row r="12">
@@ -1023,22 +1023,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.0004525860785790962</v>
+        <v>-0.9797224161140996</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.0003816079464118504</v>
+        <v>-0.7283072000158787</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.0001369910483674237</v>
+        <v>-0.2623413493463744</v>
       </c>
       <c r="E12" t="n">
-        <v>-4.73352346979284</v>
+        <v>-4.876159227282926</v>
       </c>
       <c r="F12" t="n">
-        <v>-3.72051815481646</v>
+        <v>-4.96206130207073</v>
       </c>
       <c r="G12" t="n">
-        <v>-2.388539085468819</v>
+        <v>-2.41250860811103</v>
       </c>
     </row>
     <row r="13">
@@ -1048,22 +1048,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0002259175892807094</v>
+        <v>-0.133166475902319</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0001228693969322211</v>
+        <v>-0.1527088816940722</v>
       </c>
       <c r="D13" t="n">
-        <v>7.192562823795013e-05</v>
+        <v>-0.1191809548022173</v>
       </c>
       <c r="E13" t="n">
-        <v>3.043889975170016</v>
+        <v>-1.138099081248135</v>
       </c>
       <c r="F13" t="n">
-        <v>2.018448889978462</v>
+        <v>-2.115687180844579</v>
       </c>
       <c r="G13" t="n">
-        <v>1.049637323485306</v>
+        <v>-2.077256876231234</v>
       </c>
     </row>
     <row r="14">
@@ -1073,13 +1073,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2.35274216540432</v>
+        <v>2.516190407109764</v>
       </c>
       <c r="C14" t="n">
-        <v>1.046817346714124</v>
+        <v>1.103944909441557</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8988454803369295</v>
+        <v>1.138177592902445</v>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>

</xml_diff>

<commit_message>
refactor: update run_meta.json display format for clarity; adjust Excel output handling in analysis script to ensure consistent star matrix generation
</commit_message>
<xml_diff>
--- a/outputs/05_benchmark_signals/tables_v_viii/cn/table_vi_forecast_logit.xlsx
+++ b/outputs/05_benchmark_signals/tables_v_viii/cn/table_vi_forecast_logit.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="display" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="display_stars" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -731,6 +732,323 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>5D5P</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>20D5P</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>60D5P</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MOM</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.16***</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.14**</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>STR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0.24***</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.17**</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WSTR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.17***</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.77***</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.48***</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TREND</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-0.26</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-0.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0.53***</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0.32***</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.44***</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Volat.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>-0.07</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-0.17</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-0.28***</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>52WH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>-0.07</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Dollar Volume</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>-0.86***</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>-0.68***</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-0.54***</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Zero Trade</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0.52***</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.31***</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.18***</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.21***</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>-0.27***</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.11*</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Illiq.</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>-0.98***</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>-0.73***</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>-0.26**</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lag Weekly Return</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>-0.13</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>-0.15**</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>-0.12**</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>McFadden R²</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2.52</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>